<commit_message>
Add Phase 2 Contract base model: Contract-WO link and per-contract Actual Cost
- 30_contract.xlsx: new Contract header master (CONTRACT-001/002/003)
- 20_work_order.xlsx: add nullable contract_no column (Contract 1:N WO)
- calculate_actual_total_cost_by_contract(): reuses
  calculate_actual_total_cost_by_wo() results, re-aggregated by contract_no
- validate_contract(): duplicate contract_no (reuses duplicate_keys()) and
  UNKNOWN_CONTRACT for WOs referencing a non-existent contract_no
- No Phase 1 calculation logic modified
</commit_message>
<xml_diff>
--- a/hanbit_mvp_dataset_phase1/20_work_order.xlsx
+++ b/hanbit_mvp_dataset_phase1/20_work_order.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="work_order" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="work_order" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'work_order'!$A$1:$K$21</definedName>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,6 +483,11 @@
           <t>end_date</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>contract_no</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -533,6 +538,11 @@
           <t>2026-07-01</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>CONTRACT-001</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -583,6 +593,11 @@
           <t>2026-07-02</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>CONTRACT-001</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -633,6 +648,11 @@
           <t>2026-07-03</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>CONTRACT-001</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -683,6 +703,11 @@
           <t>2026-07-04</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>CONTRACT-002</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -733,6 +758,11 @@
           <t>2026-07-05</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>CONTRACT-002</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -983,6 +1013,11 @@
           <t>2026-07-10</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>CONTRACT-002</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1133,6 +1168,11 @@
           <t>2026-07-13</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>CONTRACT-002</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1388,6 +1428,11 @@
           <t>2026-08-05</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>CONTRACT-003</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1441,6 +1486,11 @@
       <c r="K20" t="inlineStr">
         <is>
           <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>CONTRACT-003</t>
         </is>
       </c>
     </row>

</xml_diff>